<commit_message>
Update map script to filter for selected LMAs
Updated map script to include filtering to select for LMAs that drain into Lough Neagh only. Added spatial join to select only discharges within selected LMAs for updated map output.
</commit_message>
<xml_diff>
--- a/Outputs/Lough_Neagh_Treated_Discharges.xlsx
+++ b/Outputs/Lough_Neagh_Treated_Discharges.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C352"/>
+  <dimension ref="A1:C320"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5856,550 +5856,6 @@
         </is>
       </c>
     </row>
-    <row r="321">
-      <c r="A321" t="inlineStr">
-        <is>
-          <t>Ballymarlagh WwTW</t>
-        </is>
-      </c>
-      <c r="B321" t="inlineStr">
-        <is>
-          <t>Braid and Main</t>
-        </is>
-      </c>
-      <c r="C321" t="inlineStr">
-        <is>
-          <t>Deerfin Burn</t>
-        </is>
-      </c>
-    </row>
-    <row r="322">
-      <c r="A322" t="inlineStr">
-        <is>
-          <t>Ballymena WwTW</t>
-        </is>
-      </c>
-      <c r="B322" t="inlineStr">
-        <is>
-          <t>Braid and Main</t>
-        </is>
-      </c>
-      <c r="C322" t="inlineStr">
-        <is>
-          <t>River Main (Slaght)</t>
-        </is>
-      </c>
-    </row>
-    <row r="323">
-      <c r="A323" t="inlineStr">
-        <is>
-          <t>Buckna WwTW</t>
-        </is>
-      </c>
-      <c r="B323" t="inlineStr">
-        <is>
-          <t>Braid and Main</t>
-        </is>
-      </c>
-      <c r="C323" t="inlineStr">
-        <is>
-          <t>Glen Burn</t>
-        </is>
-      </c>
-    </row>
-    <row r="324">
-      <c r="A324" t="inlineStr">
-        <is>
-          <t>Cargan WwTW</t>
-        </is>
-      </c>
-      <c r="B324" t="inlineStr">
-        <is>
-          <t>Braid and Main</t>
-        </is>
-      </c>
-      <c r="C324" t="inlineStr">
-        <is>
-          <t>Glenravel Water</t>
-        </is>
-      </c>
-    </row>
-    <row r="325">
-      <c r="A325" t="inlineStr">
-        <is>
-          <t>Carnbeg WwTW</t>
-        </is>
-      </c>
-      <c r="B325" t="inlineStr">
-        <is>
-          <t>Braid and Main</t>
-        </is>
-      </c>
-      <c r="C325" t="inlineStr">
-        <is>
-          <t>River Main (Glarryford)</t>
-        </is>
-      </c>
-    </row>
-    <row r="326">
-      <c r="A326" t="inlineStr">
-        <is>
-          <t>Carnlough Road WwTW</t>
-        </is>
-      </c>
-      <c r="B326" t="inlineStr">
-        <is>
-          <t>Braid and Main</t>
-        </is>
-      </c>
-      <c r="C326" t="inlineStr">
-        <is>
-          <t>Priest's Burn</t>
-        </is>
-      </c>
-    </row>
-    <row r="327">
-      <c r="A327" t="inlineStr">
-        <is>
-          <t>Clogh WwTW</t>
-        </is>
-      </c>
-      <c r="B327" t="inlineStr">
-        <is>
-          <t>Braid and Main</t>
-        </is>
-      </c>
-      <c r="C327" t="inlineStr">
-        <is>
-          <t>Clogh River</t>
-        </is>
-      </c>
-    </row>
-    <row r="328">
-      <c r="A328" t="inlineStr">
-        <is>
-          <t>Cloghmills WwTW</t>
-        </is>
-      </c>
-      <c r="B328" t="inlineStr">
-        <is>
-          <t>Braid and Main</t>
-        </is>
-      </c>
-      <c r="C328" t="inlineStr">
-        <is>
-          <t>Cloghmills Water</t>
-        </is>
-      </c>
-    </row>
-    <row r="329">
-      <c r="A329" t="inlineStr">
-        <is>
-          <t>Connaught Road 21 ST</t>
-        </is>
-      </c>
-      <c r="B329" t="inlineStr">
-        <is>
-          <t>Braid and Main</t>
-        </is>
-      </c>
-      <c r="C329" t="inlineStr">
-        <is>
-          <t>River Main (Randalstown)</t>
-        </is>
-      </c>
-    </row>
-    <row r="330">
-      <c r="A330" t="inlineStr">
-        <is>
-          <t>Coolsythe Road 23 ST</t>
-        </is>
-      </c>
-      <c r="B330" t="inlineStr">
-        <is>
-          <t>Braid and Main</t>
-        </is>
-      </c>
-      <c r="C330" t="inlineStr">
-        <is>
-          <t>River Main (Randalstown)</t>
-        </is>
-      </c>
-    </row>
-    <row r="331">
-      <c r="A331" t="inlineStr">
-        <is>
-          <t>Craigywarren WwTW</t>
-        </is>
-      </c>
-      <c r="B331" t="inlineStr">
-        <is>
-          <t>Braid and Main</t>
-        </is>
-      </c>
-      <c r="C331" t="inlineStr">
-        <is>
-          <t>Clogh River</t>
-        </is>
-      </c>
-    </row>
-    <row r="332">
-      <c r="A332" t="inlineStr">
-        <is>
-          <t>Crankill ST</t>
-        </is>
-      </c>
-      <c r="B332" t="inlineStr">
-        <is>
-          <t>Braid and Main</t>
-        </is>
-      </c>
-      <c r="C332" t="inlineStr">
-        <is>
-          <t>Clogh River</t>
-        </is>
-      </c>
-    </row>
-    <row r="333">
-      <c r="A333" t="inlineStr">
-        <is>
-          <t>Duneany WwTW</t>
-        </is>
-      </c>
-      <c r="B333" t="inlineStr">
-        <is>
-          <t>Braid and Main</t>
-        </is>
-      </c>
-      <c r="C333" t="inlineStr">
-        <is>
-          <t>River Main (Glarryford)</t>
-        </is>
-      </c>
-    </row>
-    <row r="334">
-      <c r="A334" t="inlineStr">
-        <is>
-          <t>Dungonnell ST</t>
-        </is>
-      </c>
-      <c r="B334" t="inlineStr">
-        <is>
-          <t>Braid and Main</t>
-        </is>
-      </c>
-      <c r="C334" t="inlineStr">
-        <is>
-          <t>Glenravel Water</t>
-        </is>
-      </c>
-    </row>
-    <row r="335">
-      <c r="A335" t="inlineStr">
-        <is>
-          <t>Dunloy WwTW</t>
-        </is>
-      </c>
-      <c r="B335" t="inlineStr">
-        <is>
-          <t>Braid and Main</t>
-        </is>
-      </c>
-      <c r="C335" t="inlineStr">
-        <is>
-          <t>River Main (Dunloy)</t>
-        </is>
-      </c>
-    </row>
-    <row r="336">
-      <c r="A336" t="inlineStr">
-        <is>
-          <t>Glarryford South WwTW</t>
-        </is>
-      </c>
-      <c r="B336" t="inlineStr">
-        <is>
-          <t>Braid and Main</t>
-        </is>
-      </c>
-      <c r="C336" t="inlineStr">
-        <is>
-          <t>River Main (Cullybackey)</t>
-        </is>
-      </c>
-    </row>
-    <row r="337">
-      <c r="A337" t="inlineStr">
-        <is>
-          <t>Grove Park WwTW</t>
-        </is>
-      </c>
-      <c r="B337" t="inlineStr">
-        <is>
-          <t>Braid and Main</t>
-        </is>
-      </c>
-      <c r="C337" t="inlineStr">
-        <is>
-          <t>Kells Water (Moorfields)</t>
-        </is>
-      </c>
-    </row>
-    <row r="338">
-      <c r="A338" t="inlineStr">
-        <is>
-          <t>Killygore WwTW</t>
-        </is>
-      </c>
-      <c r="B338" t="inlineStr">
-        <is>
-          <t>Braid and Main</t>
-        </is>
-      </c>
-      <c r="C338" t="inlineStr">
-        <is>
-          <t>Clogh River</t>
-        </is>
-      </c>
-    </row>
-    <row r="339">
-      <c r="A339" t="inlineStr">
-        <is>
-          <t>Killylane ST</t>
-        </is>
-      </c>
-      <c r="B339" t="inlineStr">
-        <is>
-          <t>Braid and Main</t>
-        </is>
-      </c>
-      <c r="C339" t="inlineStr">
-        <is>
-          <t>Glenwhirry River</t>
-        </is>
-      </c>
-    </row>
-    <row r="340">
-      <c r="A340" t="inlineStr">
-        <is>
-          <t>Martinstown WwTW</t>
-        </is>
-      </c>
-      <c r="B340" t="inlineStr">
-        <is>
-          <t>Braid and Main</t>
-        </is>
-      </c>
-      <c r="C340" t="inlineStr">
-        <is>
-          <t>Clogh River</t>
-        </is>
-      </c>
-    </row>
-    <row r="341">
-      <c r="A341" t="inlineStr">
-        <is>
-          <t>Moorfields WwTW</t>
-        </is>
-      </c>
-      <c r="B341" t="inlineStr">
-        <is>
-          <t>Braid and Main</t>
-        </is>
-      </c>
-      <c r="C341" t="inlineStr">
-        <is>
-          <t>Kells Water (Moorfields)</t>
-        </is>
-      </c>
-    </row>
-    <row r="342">
-      <c r="A342" t="inlineStr">
-        <is>
-          <t>Newtown-Crommelin WwTW</t>
-        </is>
-      </c>
-      <c r="B342" t="inlineStr">
-        <is>
-          <t>Braid and Main</t>
-        </is>
-      </c>
-      <c r="C342" t="inlineStr">
-        <is>
-          <t>Skerry Water</t>
-        </is>
-      </c>
-    </row>
-    <row r="343">
-      <c r="A343" t="inlineStr">
-        <is>
-          <t>Oaklands Broughshane ST</t>
-        </is>
-      </c>
-      <c r="B343" t="inlineStr">
-        <is>
-          <t>Braid and Main</t>
-        </is>
-      </c>
-      <c r="C343" t="inlineStr">
-        <is>
-          <t>Artoges River</t>
-        </is>
-      </c>
-    </row>
-    <row r="344">
-      <c r="A344" t="inlineStr">
-        <is>
-          <t>Old Green WwTW</t>
-        </is>
-      </c>
-      <c r="B344" t="inlineStr">
-        <is>
-          <t>Braid and Main</t>
-        </is>
-      </c>
-      <c r="C344" t="inlineStr">
-        <is>
-          <t>Kells Water (Kells)</t>
-        </is>
-      </c>
-    </row>
-    <row r="345">
-      <c r="A345" t="inlineStr">
-        <is>
-          <t>Procklis WwTW</t>
-        </is>
-      </c>
-      <c r="B345" t="inlineStr">
-        <is>
-          <t>Braid and Main</t>
-        </is>
-      </c>
-      <c r="C345" t="inlineStr">
-        <is>
-          <t>River Main (Randalstown)</t>
-        </is>
-      </c>
-    </row>
-    <row r="346">
-      <c r="A346" t="inlineStr">
-        <is>
-          <t>Racavan WwTW</t>
-        </is>
-      </c>
-      <c r="B346" t="inlineStr">
-        <is>
-          <t>Braid and Main</t>
-        </is>
-      </c>
-      <c r="C346" t="inlineStr">
-        <is>
-          <t>Braid River (Broughshane)</t>
-        </is>
-      </c>
-    </row>
-    <row r="347">
-      <c r="A347" t="inlineStr">
-        <is>
-          <t>Railway View Three ST</t>
-        </is>
-      </c>
-      <c r="B347" t="inlineStr">
-        <is>
-          <t>Braid and Main</t>
-        </is>
-      </c>
-      <c r="C347" t="inlineStr">
-        <is>
-          <t>River Main (Cullybackey)</t>
-        </is>
-      </c>
-    </row>
-    <row r="348">
-      <c r="A348" t="inlineStr">
-        <is>
-          <t>Skerry View WwTW</t>
-        </is>
-      </c>
-      <c r="B348" t="inlineStr">
-        <is>
-          <t>Braid and Main</t>
-        </is>
-      </c>
-      <c r="C348" t="inlineStr">
-        <is>
-          <t>Braid River (Broughshane)</t>
-        </is>
-      </c>
-    </row>
-    <row r="349">
-      <c r="A349" t="inlineStr">
-        <is>
-          <t>Slaght WwTW</t>
-        </is>
-      </c>
-      <c r="B349" t="inlineStr">
-        <is>
-          <t>Braid and Main</t>
-        </is>
-      </c>
-      <c r="C349" t="inlineStr">
-        <is>
-          <t>River Main (Slaght)</t>
-        </is>
-      </c>
-    </row>
-    <row r="350">
-      <c r="A350" t="inlineStr">
-        <is>
-          <t>Straid Ballymena WwTW</t>
-        </is>
-      </c>
-      <c r="B350" t="inlineStr">
-        <is>
-          <t>Braid and Main</t>
-        </is>
-      </c>
-      <c r="C350" t="inlineStr">
-        <is>
-          <t>River Main (Slaght)</t>
-        </is>
-      </c>
-    </row>
-    <row r="351">
-      <c r="A351" t="inlineStr">
-        <is>
-          <t>Tullygrawley WwTW</t>
-        </is>
-      </c>
-      <c r="B351" t="inlineStr">
-        <is>
-          <t>Braid and Main</t>
-        </is>
-      </c>
-      <c r="C351" t="inlineStr">
-        <is>
-          <t>River Main (Cullybackey)</t>
-        </is>
-      </c>
-    </row>
-    <row r="352">
-      <c r="A352" t="inlineStr">
-        <is>
-          <t>Tullymore Road 43-45 ST</t>
-        </is>
-      </c>
-      <c r="B352" t="inlineStr">
-        <is>
-          <t>Braid and Main</t>
-        </is>
-      </c>
-      <c r="C352" t="inlineStr">
-        <is>
-          <t>Artoges River</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>